<commit_message>
Include AFOLU of Costa Rica model
</commit_message>
<xml_diff>
--- a/CRI/Energy/ndc_cr_30/t1_confection/A2_Extra_Inputs/A-Xtra_Scenarios.xlsx
+++ b/CRI/Energy/ndc_cr_30/t1_confection/A2_Extra_Inputs/A-Xtra_Scenarios.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28429"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29029"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\IgnacioAlfaroCorrale\Desktop\Models_running\NDC_CR\IPPU\A2_Extra_Inputs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ClimateLeadGroup\Desktop\CLG_repositories\openmodels_lac\CRI\Energy\ndc_cr_30\t1_confection\A2_Extra_Inputs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B57FEDB1-5244-497C-8C85-757C0FB244BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{14A264CB-5A31-46B6-8AD0-87EE4E148777}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-45" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Other_Params" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
   <si>
     <t>BAU</t>
   </si>
@@ -52,9 +52,6 @@
   </si>
   <si>
     <t>Timeslice</t>
-  </si>
-  <si>
-    <t>NDCincond</t>
   </si>
   <si>
     <t>CR</t>
@@ -536,14 +533,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B6"/>
-  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="18.44140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.5546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="18.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="18" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>4</v>
       </c>
@@ -551,7 +548,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>6</v>
       </c>
@@ -559,23 +556,21 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="8" t="s">
-        <v>9</v>
-      </c>
+      <c r="B3" s="8"/>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
         <v>3</v>
       </c>
@@ -583,7 +578,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="4" t="s">
         <v>8</v>
       </c>
@@ -598,26 +593,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="48eed89a-7418-4977-ae3a-838f0fac8ec5">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="416d42ac-85ec-40c4-8054-6c816fd4b6a7" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x010100C341064803B07E4F8A0204BD36BE6D07" ma:contentTypeVersion="12" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="7b6cc499061edee961e2646e4109d12b">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="48eed89a-7418-4977-ae3a-838f0fac8ec5" xmlns:ns3="416d42ac-85ec-40c4-8054-6c816fd4b6a7" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="91f4ccc8eac361410ae569a7832f6d99" ns2:_="" ns3:_="">
     <xsd:import namespace="48eed89a-7418-4977-ae3a-838f0fac8ec5"/>
@@ -818,11 +793,41 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="48eed89a-7418-4977-ae3a-838f0fac8ec5">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="416d42ac-85ec-40c4-8054-6c816fd4b6a7" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4D044BD7-CD13-4950-8112-F2F737605A34}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FF070B6D-3A26-4C62-BFDF-3A5CC28A4B40}">
   <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="48eed89a-7418-4977-ae3a-838f0fac8ec5"/>
+    <ds:schemaRef ds:uri="416d42ac-85ec-40c4-8054-6c816fd4b6a7"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -836,5 +841,12 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FF070B6D-3A26-4C62-BFDF-3A5CC28A4B40}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4D044BD7-CD13-4950-8112-F2F737605A34}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="48eed89a-7418-4977-ae3a-838f0fac8ec5"/>
+    <ds:schemaRef ds:uri="416d42ac-85ec-40c4-8054-6c816fd4b6a7"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>